<commit_message>
7.19  , move yixiaodong wrok, device placement learning
</commit_message>
<xml_diff>
--- a/论文.xlsx
+++ b/论文.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>论文题目</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -29,35 +29,51 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>Deep Learning-based Job Placement in Distributed Machine Learning Clusters,yxbao-infocom19.pdf</t>
+  </si>
+  <si>
+    <t>OptimusAn Efficient Dynamic Resource Scheduler for Deep Learning Clusters in EuroSys 2018,yhpeng-eurosys18.pdf</t>
+  </si>
+  <si>
+    <t>DRL\playing atari with deep reinforcement learning 2013.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> DQN DRL的经典模型</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Simple Statistical Gradientfollowing Algorithms for Connectionist Reinforcement Learning.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>强化学习的经典论文</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>分层放置设备</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Asynchronous Methods for Deep Reinforcement Learning.</t>
+  </si>
+  <si>
+    <t>异步方法, 讲了DRL的优化方法</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>动态分配资源RL优化, 离线监督学习预热</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>用一种无模型的深度强化学习方法来实现模型并行性，从而在一台机器中最大限度地提高给定模型的训练速度。这种方法对于深度学习集群中的资源分配还不是通用和有效的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Device Placement Optimization with Reinforcement Learning</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>A Deep Learning-driven Scheduler for Deep Learning Cluster.pdf</t>
-  </si>
-  <si>
-    <t>Deep Learning-based Job Placement in Distributed Machine Learning Clusters,yxbao-infocom19.pdf</t>
-  </si>
-  <si>
-    <t>OptimusAn Efficient Dynamic Resource Scheduler for Deep Learning Clusters in EuroSys 2018,yhpeng-eurosys18.pdf</t>
-  </si>
-  <si>
-    <t>DRL\playing atari with deep reinforcement learning 2013.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> DQN DRL的经典模型</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Simple Statistical Gradientfollowing Algorithms for Connectionist Reinforcement Learning.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>强化学习的经典论文</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>分层放置设备</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>在线动态分配资源RL优化, 离线监督学习预热</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -65,10 +81,23 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Asynchronous Methods for Deep Reinforcement Learning.</t>
-  </si>
-  <si>
-    <t>异步方法, 讲了DRL的优化方法</t>
+    <t>placement</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>resource allocation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DRL output</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>考虑干扰,DRL训练输出placement, 构建奖励NN模型提供reward预测</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>核心是精确的深度学习工作负载性能模型，利用数据模型训练的特性（如收敛性、迭代性）和参数服务器体系结构的通信模式构建的。**建模了训练速度的模型,   构建了  speed和资源的关系.**  在性能模型的基础上，设计了基于边际增益的资源分配算法和训练速度最大化的任务分配方案。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -408,49 +437,68 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A4:K20"/>
+  <dimension ref="A4:K22"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="5" max="5" width="12.58203125" customWidth="1"/>
+    <col min="6" max="6" width="10.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>0</v>
       </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" t="s">
+        <v>17</v>
+      </c>
       <c r="G4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="G5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="E6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="G7" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G10" t="s">
         <v>5</v>
-      </c>
-      <c r="G10" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G11" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -458,18 +506,26 @@
     </row>
     <row r="18" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G18" t="s">
         <v>7</v>
-      </c>
-      <c r="G18" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G20" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
first week report finished
</commit_message>
<xml_diff>
--- a/论文.xlsx
+++ b/论文.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>论文题目</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -50,10 +50,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>分层放置设备</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Asynchronous Methods for Deep Reinforcement Learning.</t>
   </si>
   <si>
@@ -73,14 +69,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>A Deep Learning-driven Scheduler for Deep Learning Cluster.pdf</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>A HIERARCHICAL MODEL FOR DEVICE PLACEMENT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>placement</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -94,6 +82,164 @@
   </si>
   <si>
     <t>考虑干扰,DRL训练输出placement, 构建奖励NN模型提供reward预测</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A HIERARCHICAL MODEL FOR DEVICE PLACEMENT2018</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Value Function Based Performance Optimization of Deep Learning Workloads 2021</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Halide</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF121212"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>与</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF121212"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>TVM</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF121212"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>将</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF121212"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>operator</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF121212"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>的表示与</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF121212"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>schedule</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF121212"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>相分离。这篇文章将</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF121212"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>schedule</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF121212"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>表示为一组优化原语（图</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF121212"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF121212"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>）的选择序列，并使用</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF121212"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Reinforcement Learning</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF121212"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>的方式进行训练。从而得到更快的搜索速度与更好的</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF121212"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>schedule</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DRL-RESOURCE ALLOCATION\A Deep Learning-driven Scheduler for Deep Learning Cluster.pdf</t>
+  </si>
+  <si>
+    <t>DRL output</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>分层放置设备 ,第一级分组,第二级placement</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -105,7 +251,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -127,6 +273,25 @@
       <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13.2"/>
+      <color rgb="FF121212"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF121212"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF121212"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="2">
@@ -150,12 +315,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -437,7 +606,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A4:K22"/>
+  <dimension ref="A4:K23"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="12.58203125" customWidth="1"/>
@@ -449,10 +618,10 @@
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G4" t="s">
         <v>1</v>
@@ -460,10 +629,13 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>14</v>
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>21</v>
       </c>
       <c r="G5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -471,10 +643,10 @@
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -482,7 +654,7 @@
         <v>3</v>
       </c>
       <c r="G7" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
@@ -495,10 +667,10 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" t="s">
         <v>9</v>
-      </c>
-      <c r="G11" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -514,27 +686,35 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G20" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G22" t="s">
-        <v>12</v>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="80.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="A5" r:id="rId1"/>
-    <hyperlink ref="A6" r:id="rId2"/>
-    <hyperlink ref="A7" r:id="rId3"/>
-    <hyperlink ref="A10" r:id="rId4"/>
+    <hyperlink ref="A6" r:id="rId1"/>
+    <hyperlink ref="A7" r:id="rId2"/>
+    <hyperlink ref="A10" r:id="rId3"/>
+    <hyperlink ref="A5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>

</xml_diff>

<commit_message>
preparing read some codes
</commit_message>
<xml_diff>
--- a/论文.xlsx
+++ b/论文.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>论文题目</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -42,10 +42,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Simple Statistical Gradientfollowing Algorithms for Connectionist Reinforcement Learning.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>强化学习的经典论文</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -78,10 +74,6 @@
   </si>
   <si>
     <t>DRL output</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>考虑干扰,DRL训练输出placement, 构建奖励NN模型提供reward预测</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -244,6 +236,18 @@
   </si>
   <si>
     <t>核心是精确的深度学习工作负载性能模型，利用数据模型训练的特性（如收敛性、迭代性）和参数服务器体系结构的通信模式构建的。**建模了训练速度的模型,   构建了  speed和资源的关系.**  在性能模型的基础上，设计了基于边际增益的资源分配算法和训练速度最大化的任务分配方案。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Simple Statistical Gradientfollowing Algorithms for Connectionist Reinforcement Learning.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>tf计算图分组然后placement</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>考虑干扰,DRL训练输出placement, 构建奖励NN模型提供reward预测</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -618,10 +622,10 @@
         <v>0</v>
       </c>
       <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
         <v>13</v>
-      </c>
-      <c r="F4" t="s">
-        <v>14</v>
       </c>
       <c r="G4" t="s">
         <v>1</v>
@@ -629,13 +633,13 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -643,10 +647,10 @@
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G6" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -654,7 +658,7 @@
         <v>3</v>
       </c>
       <c r="G7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
@@ -667,10 +671,10 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G11" t="s">
         <v>8</v>
-      </c>
-      <c r="G11" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -678,34 +682,37 @@
     </row>
     <row r="18" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G18" t="s">
         <v>6</v>
-      </c>
-      <c r="G18" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>17</v>
+        <v>15</v>
+      </c>
+      <c r="E20" t="s">
+        <v>23</v>
       </c>
       <c r="G20" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G22" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="80.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
i am writing input and output for my first idea
</commit_message>
<xml_diff>
--- a/论文.xlsx
+++ b/论文.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>论文题目</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -81,12 +81,23 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Value Function Based Performance Optimization of Deep Learning Workloads 2021</t>
+    <t>DRL-RESOURCE ALLOCATION\A Deep Learning-driven Scheduler for Deep Learning Cluster.pdf</t>
+  </si>
+  <si>
+    <t>DRL output</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>核心是精确的深度学习工作负载性能模型，利用数据模型训练的特性（如收敛性、迭代性）和参数服务器体系结构的通信模式构建的。**建模了训练速度的模型,   构建了  speed和资源的关系.**  在性能模型的基础上，设计了基于边际增益的资源分配算法和训练速度最大化的任务分配方案。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>考虑干扰,DRL训练输出placement, 构建奖励NN模型提供reward预测</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <r>
-      <t>Halide</t>
+      <t>DQN,</t>
     </r>
     <r>
       <rPr>
@@ -96,7 +107,7 @@
         <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t>与</t>
+      <t>用</t>
     </r>
     <r>
       <rPr>
@@ -105,7 +116,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>TVM</t>
+      <t xml:space="preserve"> DNN</t>
     </r>
     <r>
       <rPr>
@@ -115,127 +126,20 @@
         <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t>将</t>
+      <t>来拟合最佳action函数Q(s,a)</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF121212"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>operator</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF121212"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>的表示与</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF121212"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>schedule</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF121212"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>相分离。这篇文章将</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF121212"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>schedule</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF121212"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>表示为一组优化原语（图</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF121212"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF121212"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>）的选择序列，并使用</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF121212"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Reinforcement Learning</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF121212"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>的方式进行训练。从而得到更快的搜索速度与更好的</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF121212"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>schedule</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DRL-RESOURCE ALLOCATION\A Deep Learning-driven Scheduler for Deep Learning Cluster.pdf</t>
-  </si>
-  <si>
-    <t>DRL output</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>分层放置设备 ,第一级分组,第二级placement</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>核心是精确的深度学习工作负载性能模型，利用数据模型训练的特性（如收敛性、迭代性）和参数服务器体系结构的通信模式构建的。**建模了训练速度的模型,   构建了  speed和资源的关系.**  在性能模型的基础上，设计了基于边际增益的资源分配算法和训练速度最大化的任务分配方案。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Human-level control through deep reinforcement learning2015</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>分层的论文</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>tf计算图operation分组然后placement</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -243,11 +147,41 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>tf计算图分组然后placement</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>考虑干扰,DRL训练输出placement, 构建奖励NN模型提供reward预测</t>
+    <t>强化学习的论文</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Kulkarni, Tejas D., et al. "Hierarchical deep reinforcement learning: Integrating temporal abstraction and intrinsic motivation." Advances in neural information processing systems. 2016.</t>
+  </si>
+  <si>
+    <t>分层放置设备 ,第一级FNN分组,第二级用LSTMplacement</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>分层强化学习,一级meta controller ,下一级controller,都是用DQN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>问题</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>做了太多工程优化,没有和其他对比</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Learning Multi-Level Hierachies with Hindsight</t>
+  </si>
+  <si>
+    <t>HRL中一般分多个层次进行控制，上下层同时训练的时候会出现non-stationary的问题，也就是下层的policy改变时会影响上层的transition，因此可能原来能达到某个goal，但现在达不到了，对学习造成很大影响。本文提出的做法是，假设下层的policy已经是最优，就不会因为下层policy的变化而影响上层，那么如何使还没有达到最优的下层policy看上去最优呢？通过HER来实现。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>每一层的reward</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>meta-controller 选择一个goal, 里面的controller选择action,只有goal被达到了, meta-controller才选择下一个goal</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -279,12 +213,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="13.2"/>
-      <color rgb="FF121212"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color rgb="FF121212"/>
       <name val="Arial"/>
@@ -296,6 +224,12 @@
       <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF646464"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -325,10 +259,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -610,7 +542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A4:K23"/>
+  <dimension ref="A4:K28"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="12.58203125" customWidth="1"/>
@@ -630,13 +562,16 @@
       <c r="G4" t="s">
         <v>1</v>
       </c>
+      <c r="J4" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G5" t="s">
         <v>9</v>
@@ -650,7 +585,7 @@
         <v>14</v>
       </c>
       <c r="G6" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -658,72 +593,112 @@
         <v>3</v>
       </c>
       <c r="G7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G10" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>7</v>
-      </c>
-      <c r="G11" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="K13" s="2"/>
     </row>
-    <row r="18" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>11</v>
+      </c>
+      <c r="G16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>7</v>
+      </c>
+      <c r="G19" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G20" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
         <v>22</v>
       </c>
-      <c r="G18" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="E24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
         <v>15</v>
       </c>
-      <c r="E20" t="s">
+      <c r="D25" t="s">
         <v>23</v>
       </c>
-      <c r="G20" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>11</v>
-      </c>
-      <c r="G22" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="80.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>17</v>
-      </c>
+      <c r="G25" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E26" t="s">
+        <v>34</v>
+      </c>
+      <c r="G26" t="s">
+        <v>28</v>
+      </c>
+      <c r="J26" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="A6" r:id="rId1"/>
     <hyperlink ref="A7" r:id="rId2"/>
-    <hyperlink ref="A10" r:id="rId3"/>
+    <hyperlink ref="A20" r:id="rId3"/>
     <hyperlink ref="A5" r:id="rId4"/>
+    <hyperlink ref="A26" r:id="rId5" display="https://link.zhihu.com/?target=http%3A//papers.nips.cc/paper/6233-hierarchical-deep-reinforcement-learning-integrating-temporal-abstraction-and-intrinsic-motivation.pdf"/>
+    <hyperlink ref="A27" r:id="rId6" display="https://link.zhihu.com/?target=http%3A//arxiv.org/abs/1712.00948v4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
I am working about reward
</commit_message>
<xml_diff>
--- a/论文.xlsx
+++ b/论文.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="RL思想 " sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
   <si>
     <t>论文题目</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -158,30 +159,61 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>问题</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Learning Multi-Level Hierachies with Hindsight</t>
+  </si>
+  <si>
+    <t>每一层的reward</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>meta-controller 选择一个goal, 里面的controller选择action,只有goal被达到了, meta-controller才选择下一个goal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>做了太多工程优化,没有和其他对比</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>分层强化学习,一级meta controller ,下一级controller,都是用DQN</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>问题</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>做了太多工程优化,没有和其他对比</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Learning Multi-Level Hierachies with Hindsight</t>
-  </si>
-  <si>
-    <t>HRL中一般分多个层次进行控制，上下层同时训练的时候会出现non-stationary的问题，也就是下层的policy改变时会影响上层的transition，因此可能原来能达到某个goal，但现在达不到了，对学习造成很大影响。本文提出的做法是，假设下层的policy已经是最优，就不会因为下层policy的变化而影响上层，那么如何使还没有达到最优的下层policy看上去最优呢？通过HER来实现。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>每一层的reward</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>meta-controller 选择一个goal, 里面的controller选择action,只有goal被达到了, meta-controller才选择下一个goal</t>
+    <t>实现了3层的连续空间, HRL中一般分多个层次进行控制，上下层同时训练的时候会出现non-stationary的问题，也就是下层的policy改变时会影响上层的transition，因此可能原来能达到某个goal，但现在达不到了，对学习造成很大影响。本文提出的做法是，假设下层的policy已经是最优，就不会因为下层policy的变化而影响上层，那么如何使还没有达到最优的下层policy看上去最优呢？通过HER来实现。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://luthuli.cs.uiuc.edu/~daf/courses/games/AIpapers/ng99policy.pdf</t>
+  </si>
+  <si>
+    <t>论文</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>思想</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reward Shaping Invariance 估计到位置, 这样收敛的快</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>reward稀疏</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hindsight Experience Replay2017</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>奖励稀疏</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>对于每一个transition都去计算一下如果换作其他目标该transition会怎样。st, at,st+1 都是不变的，只需要重新计算一下新目标g' 下的奖励.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -189,7 +221,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -231,6 +263,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF121212"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -253,7 +291,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -261,6 +299,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -563,7 +602,7 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -649,7 +688,7 @@
         <v>22</v>
       </c>
       <c r="E24" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
@@ -668,21 +707,21 @@
         <v>26</v>
       </c>
       <c r="E26" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G26" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="J26" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G27" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
@@ -701,4 +740,52 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A5:E8"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="12.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="17.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
leraning a3c policy gradient
</commit_message>
<xml_diff>
--- a/论文.xlsx
+++ b/论文.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="RL思想 " sheetId="2" r:id="rId2"/>
+    <sheet name="RL codes" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="57">
   <si>
     <t>论文题目</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -47,21 +48,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Asynchronous Methods for Deep Reinforcement Learning.</t>
-  </si>
-  <si>
     <t>异步方法, 讲了DRL的优化方法</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>动态分配资源RL优化, 离线监督学习预热</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>用一种无模型的深度强化学习方法来实现模型并行性，从而在一台机器中最大限度地提高给定模型的训练速度。这种方法对于深度学习集群中的资源分配还不是通用和有效的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Device Placement Optimization with Reinforcement Learning</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -78,22 +68,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>A HIERARCHICAL MODEL FOR DEVICE PLACEMENT2018</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DRL-RESOURCE ALLOCATION\A Deep Learning-driven Scheduler for Deep Learning Cluster.pdf</t>
-  </si>
-  <si>
-    <t>DRL output</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>核心是精确的深度学习工作负载性能模型，利用数据模型训练的特性（如收敛性、迭代性）和参数服务器体系结构的通信模式构建的。**建模了训练速度的模型,   构建了  speed和资源的关系.**  在性能模型的基础上，设计了基于边际增益的资源分配算法和训练速度最大化的任务分配方案。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>考虑干扰,DRL训练输出placement, 构建奖励NN模型提供reward预测</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -144,76 +119,278 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>强化学习的论文</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Kulkarni, Tejas D., et al. "Hierarchical deep reinforcement learning: Integrating temporal abstraction and intrinsic motivation." Advances in neural information processing systems. 2016.</t>
+  </si>
+  <si>
+    <t>问题</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Learning Multi-Level Hierachies with Hindsight</t>
+  </si>
+  <si>
+    <t>每一层的reward</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>meta-controller 选择一个goal, 里面的controller选择action,只有goal被达到了, meta-controller才选择下一个goal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>做了太多工程优化,没有和其他对比</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>实现了3层的连续空间, HRL中一般分多个层次进行控制，上下层同时训练的时候会出现non-stationary的问题，也就是下层的policy改变时会影响上层的transition，因此可能原来能达到某个goal，但现在达不到了，对学习造成很大影响。本文提出的做法是，假设下层的policy已经是最优，就不会因为下层policy的变化而影响上层，那么如何使还没有达到最优的下层policy看上去最优呢？通过HER来实现。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>论文</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>思想</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reward Shaping Invariance 估计到位置, 这样收敛的快</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>reward稀疏</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>奖励稀疏</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>对于每一个transition都去计算一下如果换作其他目标该transition会怎样。st, at,st+1 都是不变的，只需要重新计算一下新目标g' 下的奖励.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://luthuli.cs.uiuc.edu/~daf/courses/games/AIpapers/ng99policy.pdf</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">hierarchy本身就是一种解决reward稀疏的方法, 比如推荐先推荐大类然后推荐细分物品. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Neural Adaptive Video Streaming with Pensieve</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>我需要找一个简单的demo搞懂框架, 运行.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://github.com/mveres01/pytorch-drl4vrp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hindsight Experience Replay2017</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>分层强化学习,一级meta controller ,下一级controller,都是用DQN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">
+</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>分层放置设备 ,第一级FNN分组,第二级用LSTMplacement</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>用一种无模型的深度强化学习方法来实现模型并行性，从而在一台机器中最大限度地提高给定模型的训练速度。这种方法对于深度学习集群中的资源分配还不是通用和有效的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">harmony的实现参考了这个,用RL实现视频算法/不需要预先规划模型和假设,
+代码, 她里面好像已经有视频了, 首先setup 通过下载了大量包. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A HIERARCHICAL MODEL FOR DEVICE PLACEMENT2018</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Asynchronous Methods for Deep Reinforcement Learning.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>Simple Statistical Gradientfollowing Algorithms for Connectionist Reinforcement Learning.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>强化学习的论文</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Kulkarni, Tejas D., et al. "Hierarchical deep reinforcement learning: Integrating temporal abstraction and intrinsic motivation." Advances in neural information processing systems. 2016.</t>
-  </si>
-  <si>
-    <t>分层放置设备 ,第一级FNN分组,第二级用LSTMplacement</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>问题</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Learning Multi-Level Hierachies with Hindsight</t>
-  </si>
-  <si>
-    <t>每一层的reward</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>meta-controller 选择一个goal, 里面的controller选择action,只有goal被达到了, meta-controller才选择下一个goal</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>做了太多工程优化,没有和其他对比</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>分层强化学习,一级meta controller ,下一级controller,都是用DQN</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>实现了3层的连续空间, HRL中一般分多个层次进行控制，上下层同时训练的时候会出现non-stationary的问题，也就是下层的policy改变时会影响上层的transition，因此可能原来能达到某个goal，但现在达不到了，对学习造成很大影响。本文提出的做法是，假设下层的policy已经是最优，就不会因为下层policy的变化而影响上层，那么如何使还没有达到最优的下层policy看上去最优呢？通过HER来实现。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://luthuli.cs.uiuc.edu/~daf/courses/games/AIpapers/ng99policy.pdf</t>
-  </si>
-  <si>
-    <t>论文</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>思想</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Reward Shaping Invariance 估计到位置, 这样收敛的快</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>reward稀疏</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Hindsight Experience Replay2017</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>奖励稀疏</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>对于每一个transition都去计算一下如果换作其他目标该transition会怎样。st, at,st+1 都是不变的，只需要重新计算一下新目标g' 下的奖励.</t>
+    <t>DRL-RESOURCE ALLOCATION\A Deep Learning-driven Scheduler for Deep Learning Cluster.pdf</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>动态分配资源RL优化, 离线监督学习预热</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>考虑干扰,DRL训练输出placement, 构建奖励NN模型提供reward预测</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DRL output</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI4Finance-LLC/ElegantRL: Lightweight, efficient and stable implementations of deep reinforcement learning algorithms using PyTorch. 🔥 (github.com)</t>
+  </si>
+  <si>
+    <t>这个就是一个简单的框架</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ElegantRL: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF121212"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>基于</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF121212"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>PyTorch</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF121212"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>的轻量</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF121212"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF121212"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>高效</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF121212"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF121212"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>稳定的深度强化学习框架</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF121212"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF121212"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>曾伊言的文章</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF121212"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF121212"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>知乎</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF121212"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> https://zhuanlan.zhihu.com/p/358560363</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Deep Reinforcement Learning for Solving the Vehicle Routing Problem</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RNN 叠加注意力机制</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>可以学习它的DRL , 策略梯度算法,  a3c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>V. Mnih, A. P. Badia, M. Mirza, A. Graves, T. Lillicrap, T. Harley, D. Silver, and K. Kavukcuoglu, “Asynchronous Methods for Deep Reinforcement Learning,” in Proc. of ICML, 2016.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>实现了快速训练,a3c</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -221,7 +398,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -269,6 +446,19 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF121212"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF121212"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -291,7 +481,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -300,6 +490,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -593,27 +784,27 @@
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G4" t="s">
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="F5" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G5" t="s">
-        <v>9</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
@@ -621,10 +812,10 @@
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="G6" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
@@ -632,7 +823,7 @@
         <v>3</v>
       </c>
       <c r="G7" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -640,20 +831,20 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G16" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="G17" t="s">
         <v>6</v>
@@ -661,18 +852,18 @@
     </row>
     <row r="18" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>43</v>
+      </c>
+      <c r="G19" t="s">
         <v>7</v>
-      </c>
-      <c r="G19" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
@@ -685,43 +876,43 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E24" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>15</v>
+        <v>42</v>
       </c>
       <c r="D25" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G25" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E26" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="G26" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="J26" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="G27" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
@@ -744,48 +935,126 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A5:E8"/>
+  <dimension ref="A3:E11"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="12.1640625" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>32</v>
+      </c>
+    </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
         <v>28</v>
       </c>
-      <c r="E5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" t="s">
-        <v>39</v>
-      </c>
       <c r="E7" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="E8" t="s">
-        <v>42</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A7" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A3:G24"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="6" max="6" width="30.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F16" t="s">
+        <v>54</v>
+      </c>
+      <c r="G16" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24" spans="6:6" ht="28" x14ac:dyDescent="0.3">
+      <c r="F24" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="C16" r:id="rId1"/>
+    <hyperlink ref="A4" r:id="rId2" display="https://github.com/AI4Finance-LLC/ElegantRL"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
7.31 , half an month
</commit_message>
<xml_diff>
--- a/论文.xlsx
+++ b/论文.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
   <si>
     <t>论文题目</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -29,9 +29,6 @@
   <si>
     <t>key idea</t>
     <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Deep Learning-based Job Placement in Distributed Machine Learning Clusters,yxbao-infocom19.pdf</t>
   </si>
   <si>
     <t>OptimusAn Efficient Dynamic Resource Scheduler for Deep Learning Clusters in EuroSys 2018,yhpeng-eurosys18.pdf</t>
@@ -181,10 +178,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Neural Adaptive Video Streaming with Pensieve</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>我需要找一个简单的demo搞懂框架, 运行.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -228,10 +221,6 @@
   </si>
   <si>
     <t>Simple Statistical Gradientfollowing Algorithms for Connectionist Reinforcement Learning.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DRL-RESOURCE ALLOCATION\A Deep Learning-driven Scheduler for Deep Learning Cluster.pdf</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -391,6 +380,36 @@
   </si>
   <si>
     <t>实现了快速训练,a3c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MorvanZhou/pytorch-A3C: Simple A3C implementation with pytorch + multiprocessing (github.com)</t>
+  </si>
+  <si>
+    <t>pytorch实现a3c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Neural Adaptive Video Streaming with Pensieve</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DRL-RESOURCE ALLOCATION\A Deep Learning-driven Scheduler for Deep Learning Cluster.pdf</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Deep Learning-based Job Placement in Distributed Machine Learning Clusters,yxbao-infocom19.pdf</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://github.com/datawhalechina/easy-rl</t>
+  </si>
+  <si>
+    <t>传统RL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://datawhalechina.github.io/easy-rl/#/</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -507,6 +526,121 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>146050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="图片 1" descr="C:\Users\12638\AppData\Roaming\Tencent\QQ\Temp\%W@GJ$ACOF(TYDYECOKVDYB.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="2311400"/>
+          <a:ext cx="190500" cy="146050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>146050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="图片 2" descr="C:\Users\12638\AppData\Roaming\Tencent\QQ\Temp\%W@GJ$ACOF(TYDYECOKVDYB.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="2641600" y="2311400"/>
+          <a:ext cx="190500" cy="146050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -784,46 +918,46 @@
         <v>0</v>
       </c>
       <c r="E4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s">
         <v>9</v>
-      </c>
-      <c r="F4" t="s">
-        <v>10</v>
       </c>
       <c r="G4" t="s">
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="F5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>2</v>
+        <v>58</v>
       </c>
       <c r="E6" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
@@ -831,88 +965,88 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G16" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G17" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G19" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G20" t="s">
         <v>4</v>
-      </c>
-      <c r="G20" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E24" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D25" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G25" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E26" t="s">
+        <v>21</v>
+      </c>
+      <c r="G26" t="s">
+        <v>35</v>
+      </c>
+      <c r="J26" t="s">
         <v>22</v>
-      </c>
-      <c r="G26" t="s">
-        <v>37</v>
-      </c>
-      <c r="J26" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G27" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
@@ -943,48 +1077,48 @@
   <sheetData>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" t="s">
         <v>25</v>
-      </c>
-      <c r="D5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" t="s">
         <v>29</v>
-      </c>
-      <c r="E8" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E11" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1007,45 +1141,64 @@
   <sheetData>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F4" t="s">
-        <v>50</v>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F14" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F16" t="s">
+        <v>51</v>
+      </c>
+      <c r="G16" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C17" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="G16" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="24" spans="6:6" ht="28" x14ac:dyDescent="0.3">
+      <c r="F17" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="24" spans="3:6" ht="28" x14ac:dyDescent="0.3">
       <c r="F24" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1053,8 +1206,11 @@
   <hyperlinks>
     <hyperlink ref="C16" r:id="rId1"/>
     <hyperlink ref="A4" r:id="rId2" display="https://github.com/AI4Finance-LLC/ElegantRL"/>
+    <hyperlink ref="C17" r:id="rId3" display="https://github.com/MorvanZhou/pytorch-A3C"/>
+    <hyperlink ref="E14" r:id="rId4" location="/"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
+  <drawing r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
I am study ing about use which network? FNN or attention or LSTM? and I need to implment the env in DL2
</commit_message>
<xml_diff>
--- a/论文.xlsx
+++ b/论文.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="70">
   <si>
     <t>论文题目</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -413,19 +413,34 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>AWAC  nair 2020  . 用离线数据集加速online</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hierarchical Reinforcement Learning | Papers With Code</t>
+  </si>
+  <si>
+    <t>有一些实现分层RL的算法.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AAAI ,WWW , ICLR, ICML, IJCAI,NeurlPS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DBLP数据库</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gandiva: Introspective Cluster Scheduling for Deep Learning</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t xml:space="preserve">accelerating online reinforcement learning with offline datasets </t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>AWAC  nair 2020  . 用离线数据集加速online</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Hierarchical Reinforcement Learning | Papers With Code</t>
-  </si>
-  <si>
-    <t>有一些实现分层RL的算法.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+    <t>Spotlight: Optimizing Device Placement for Training Deep Neural Networks</t>
   </si>
 </sst>
 </file>
@@ -921,14 +936,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A4:K28"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K28"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="5" max="5" width="12.58203125" customWidth="1"/>
+    <col min="5" max="5" width="12.625" customWidth="1"/>
     <col min="6" max="6" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -945,7 +970,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>57</v>
       </c>
@@ -956,7 +981,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>58</v>
       </c>
@@ -967,7 +992,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>2</v>
       </c>
@@ -975,15 +1000,25 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="K13" s="2"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>7</v>
       </c>
@@ -991,7 +1026,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>42</v>
       </c>
@@ -999,7 +1034,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" ht="29.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>13</v>
       </c>
@@ -1007,7 +1042,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -1015,7 +1050,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>3</v>
       </c>
@@ -1023,15 +1058,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>68</v>
+      </c>
+      <c r="G21" t="s">
         <v>62</v>
       </c>
-      <c r="G21" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>14</v>
       </c>
@@ -1039,7 +1074,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>40</v>
       </c>
@@ -1050,7 +1085,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>17</v>
       </c>
@@ -1064,7 +1099,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>19</v>
       </c>
@@ -1072,7 +1107,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="4"/>
     </row>
   </sheetData>
@@ -1093,17 +1128,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A3:E11"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="12.1640625" customWidth="1"/>
+    <col min="4" max="4" width="12.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -1114,7 +1149,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>30</v>
       </c>
@@ -1125,7 +1160,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="18" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>34</v>
       </c>
@@ -1136,7 +1171,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>52</v>
       </c>
@@ -1157,17 +1192,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A3:G24"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="6" max="6" width="30.83203125" customWidth="1"/>
+    <col min="6" max="6" width="30.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>46</v>
       </c>
@@ -1178,7 +1213,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>59</v>
       </c>
@@ -1189,7 +1224,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>56</v>
       </c>
@@ -1197,7 +1232,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>49</v>
       </c>
@@ -1211,7 +1246,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C17" s="1" t="s">
         <v>54</v>
       </c>
@@ -1219,15 +1254,15 @@
         <v>55</v>
       </c>
     </row>
-    <row r="18" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C18" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F18" t="s">
         <v>64</v>
       </c>
-      <c r="F18" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="24" spans="3:6" ht="28" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="3:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="F24" s="2" t="s">
         <v>36</v>
       </c>

</xml_diff>

<commit_message>
I read two papers , I am reading osid
</commit_message>
<xml_diff>
--- a/论文.xlsx
+++ b/论文.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="78">
   <si>
     <t>论文题目</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -441,13 +441,43 @@
   </si>
   <si>
     <t>Spotlight: Optimizing Device Placement for Training Deep Neural Networks</t>
+  </si>
+  <si>
+    <t>Shulman 等Proximal policy optimization algorithms.，2017</t>
+  </si>
+  <si>
+    <t>策略梯度优化方法</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>还可以参考Heess, N., TB, D., Sriram, S., Merel, J., Wayne, G., Tassa, Y., Erez, T., Wang, Z., Eslami, A., and Riedmiller, M. Emergence of locomotion behaviours in rich environments. In arXiv:1707.02286, 2017.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Heterogeneity-Aware Cluster Scheduling Policies for Deep Learning Workloads  Nov2020</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>斯坦福大学刊登在osdi20顶会</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://github.com/dgriff777/rl_a3c_pytorch</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A3C LSTM Atari with Pytorch plus A3G design</t>
+  </si>
+  <si>
+    <t>代码地址https://github.com/stanford-futuredata/gavel</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -508,6 +538,18 @@
       <family val="3"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF24292E"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -530,7 +572,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -540,6 +582,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1011,6 +1055,15 @@
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E13" t="s">
+        <v>74</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>77</v>
+      </c>
       <c r="K13" s="2"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
@@ -1064,6 +1117,17 @@
       </c>
       <c r="G21" t="s">
         <v>62</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15" x14ac:dyDescent="0.2">
+      <c r="A22" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="G22" t="s">
+        <v>71</v>
+      </c>
+      <c r="J22" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
@@ -1119,9 +1183,10 @@
     <hyperlink ref="A5" r:id="rId4"/>
     <hyperlink ref="A26" r:id="rId5" display="https://link.zhihu.com/?target=http%3A//papers.nips.cc/paper/6233-hierarchical-deep-reinforcement-learning-integrating-temporal-abstraction-and-intrinsic-motivation.pdf"/>
     <hyperlink ref="A27" r:id="rId6" display="https://link.zhihu.com/?target=http%3A//arxiv.org/abs/1712.00948v4"/>
+    <hyperlink ref="I13" r:id="rId7" display="https://github.com/stanford-futuredata/gavel"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
 
@@ -1262,6 +1327,14 @@
         <v>64</v>
       </c>
     </row>
+    <row r="21" spans="3:6" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="C21" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>76</v>
+      </c>
+    </row>
     <row r="24" spans="3:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="F24" s="2" t="s">
         <v>36</v>
@@ -1275,9 +1348,10 @@
     <hyperlink ref="C17" r:id="rId3" display="https://github.com/MorvanZhou/pytorch-A3C"/>
     <hyperlink ref="E14" r:id="rId4" location="/"/>
     <hyperlink ref="C18" r:id="rId5" display="https://paperswithcode.com/task/hierarchical-reinforcement-learning"/>
+    <hyperlink ref="C21" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
-  <drawing r:id="rId7"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
+  <drawing r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
doing  agent cluster find way to use
</commit_message>
<xml_diff>
--- a/论文.xlsx
+++ b/论文.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="87">
   <si>
     <t>论文题目</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -116,10 +116,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>强化学习的论文</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Kulkarni, Tejas D., et al. "Hierarchical deep reinforcement learning: Integrating temporal abstraction and intrinsic motivation." Advances in neural information processing systems. 2016.</t>
   </si>
   <si>
@@ -200,10 +196,6 @@
   </si>
   <si>
     <t>分层放置设备 ,第一级FNN分组,第二级用LSTMplacement</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>用一种无模型的深度强化学习方法来实现模型并行性，从而在一台机器中最大限度地提高给定模型的训练速度。这种方法对于深度学习集群中的资源分配还不是通用和有效的</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -446,34 +438,70 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>还可以参考Heess, N., TB, D., Sriram, S., Merel, J., Wayne, G., Tassa, Y., Erez, T., Wang, Z., Eslami, A., and Riedmiller, M. Emergence of locomotion behaviours in rich environments. In arXiv:1707.02286, 2017.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Heterogeneity-Aware Cluster Scheduling Policies for Deep Learning Workloads  Nov2020</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>https://github.com/dgriff777/rl_a3c_pytorch</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A3C LSTM Atari with Pytorch plus A3G design</t>
+  </si>
+  <si>
+    <t>代码地址https://github.com/stanford-futuredata/gavel</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>这个就是一个简单的框架,evalutor类可以保存配置和每个episode的奖励</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>多智能体可以看Rllib,  deep di lab, github用户starry的MARL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>用一种无模型的深度强化学习方法来实现模型并行性，从而在一台机器中最大限度地提高给定模型的训练速度。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>这种方法对于深度学习集群中的资源分配还不是通用和有效的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>斯坦福大学刊登在osdi20顶会</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>https://github.com/dgriff777/rl_a3c_pytorch</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>A3C LSTM Atari with Pytorch plus A3G design</t>
-  </si>
-  <si>
-    <t>代码地址https://github.com/stanford-futuredata/gavel</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>这个就是一个简单的框架,evalutor类可以保存配置和每个episode的奖励</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>多智能体可以看Rllib,  deep di lab, github用户starry的MARL</t>
+    <t>Pollux: Co-adaptive Cluster Scheduling for Goodput-Optimized Deep Learning</t>
+  </si>
+  <si>
+    <t>是</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Low-latency Job Scheduling with Preemption for the Development of Deep Learning   OpML19 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.usenix.org/system/files/opml19papers-yabuuchi.pdf</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.usenix.org/sites/default/files/conference/protected-files/opml19_slides_yabuuchi.pdf</t>
+  </si>
+  <si>
+    <t>左边是pdf右边是ppt</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">trail and error (TE) 作业的高效作业调度是深度学习项目中的一个具有挑战性的问题。 不幸的是，迄今为止，现有的作业调度程序没有为 TE 和best-effort (BE) 作业的混合调度提供良好的平衡，或者它们最多只能在有限的情况下处理混合。 为了填补这一空白，我们提出了一种算法，该算法通过有选择地抢占 BE 作业来有效地调度 TE 和 BE 作业，这些作业可以在时机成熟时毫不延迟地恢复。 </t>
+  </si>
+  <si>
+    <t>做了一些抢占的调度, 看了和DRL没啥关系就略过了.</t>
+  </si>
+  <si>
+    <t>和目前主题无关但是有关优化调度的论文</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -481,7 +509,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -554,6 +582,13 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color rgb="FF5B808D"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -576,7 +611,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -588,6 +623,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -984,7 +1020,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="12.625" customWidth="1"/>
@@ -993,12 +1029,12 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
@@ -1015,29 +1051,29 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F5" t="s">
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
@@ -1050,144 +1086,113 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>69</v>
+      </c>
+      <c r="E13" t="s">
+        <v>77</v>
+      </c>
+      <c r="I13" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E13" t="s">
-        <v>73</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>76</v>
-      </c>
       <c r="K13" s="2"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>7</v>
-      </c>
-      <c r="G16" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G17" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="29.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>41</v>
-      </c>
-      <c r="G19" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G20" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>67</v>
-      </c>
-      <c r="G21" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="15" x14ac:dyDescent="0.2">
-      <c r="A22" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="G22" t="s">
-        <v>70</v>
-      </c>
-      <c r="J22" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>78</v>
+      </c>
+      <c r="F14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>14</v>
       </c>
       <c r="E24" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D25" t="s">
         <v>15</v>
       </c>
       <c r="G25" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E26" t="s">
+        <v>20</v>
+      </c>
+      <c r="G26" t="s">
+        <v>34</v>
+      </c>
+      <c r="J26" t="s">
         <v>21</v>
       </c>
-      <c r="G26" t="s">
-        <v>35</v>
-      </c>
-      <c r="J26" t="s">
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G27" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G27" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="4"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="15" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>80</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="H31" t="s">
+        <v>83</v>
+      </c>
+      <c r="J31" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="L31" s="7" t="s">
+        <v>85</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="A6" r:id="rId1"/>
     <hyperlink ref="A7" r:id="rId2"/>
-    <hyperlink ref="A20" r:id="rId3"/>
-    <hyperlink ref="A5" r:id="rId4"/>
-    <hyperlink ref="A26" r:id="rId5" display="https://link.zhihu.com/?target=http%3A//papers.nips.cc/paper/6233-hierarchical-deep-reinforcement-learning-integrating-temporal-abstraction-and-intrinsic-motivation.pdf"/>
-    <hyperlink ref="A27" r:id="rId6" display="https://link.zhihu.com/?target=http%3A//arxiv.org/abs/1712.00948v4"/>
-    <hyperlink ref="I13" r:id="rId7" display="https://github.com/stanford-futuredata/gavel"/>
+    <hyperlink ref="A5" r:id="rId3"/>
+    <hyperlink ref="A26" r:id="rId4" display="https://link.zhihu.com/?target=http%3A//papers.nips.cc/paper/6233-hierarchical-deep-reinforcement-learning-integrating-temporal-abstraction-and-intrinsic-motivation.pdf"/>
+    <hyperlink ref="A27" r:id="rId5" display="https://link.zhihu.com/?target=http%3A//arxiv.org/abs/1712.00948v4"/>
+    <hyperlink ref="I13" r:id="rId6" display="https://github.com/stanford-futuredata/gavel"/>
+    <hyperlink ref="F31" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
@@ -1196,65 +1201,125 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:E11"/>
+  <dimension ref="A3:J22"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="12.125" customWidth="1"/>
+    <col min="10" max="10" width="12.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" t="s">
         <v>24</v>
       </c>
-      <c r="D5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="J5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="J7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+      <c r="J8" t="s">
         <v>27</v>
       </c>
-      <c r="E7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E11" t="s">
-        <v>52</v>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="29.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="G15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G16" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>65</v>
+      </c>
+      <c r="G17" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="15" x14ac:dyDescent="0.2">
+      <c r="A18" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="G18" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>7</v>
+      </c>
+      <c r="G22" t="s">
+        <v>75</v>
+      </c>
+      <c r="J22" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="A7" r:id="rId1"/>
+    <hyperlink ref="A16" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -1268,85 +1333,85 @@
   <sheetData>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F4" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F5" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="F14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F16" t="s">
         <v>48</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F16" t="s">
-        <v>50</v>
-      </c>
       <c r="G16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C17" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F17" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C18" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F18" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" spans="3:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="C21" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="24" spans="3:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="F24" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finished PS  communication , doing allreduce ring communication thourghput
</commit_message>
<xml_diff>
--- a/论文.xlsx
+++ b/论文.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="92">
   <si>
     <t>论文题目</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -517,6 +517,14 @@
 2 对接口的传输速度进行实验探究，并采取最后的数据传输策略；
 3 提出新的方案使得GPU-CPU能更好的协同工作；
 4 测试；</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://jcf94.com/2017/12/20/2017-12-20-distributeddl/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2018年之前的分布式机器学习综述</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1149,6 +1157,14 @@
         <v>89</v>
       </c>
     </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="G26" t="s">
+        <v>91</v>
+      </c>
+    </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="4"/>
     </row>
@@ -1185,9 +1201,10 @@
     <hyperlink ref="A5" r:id="rId3"/>
     <hyperlink ref="I13" r:id="rId4" display="https://github.com/stanford-futuredata/gavel"/>
     <hyperlink ref="F31" r:id="rId5"/>
+    <hyperlink ref="A26" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
professor wants me to implment and give experiment results. But I implement this program very slow. Research is difficult
</commit_message>
<xml_diff>
--- a/论文.xlsx
+++ b/论文.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="96">
   <si>
     <t>论文题目</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -532,6 +532,14 @@
   </si>
   <si>
     <t>医疗资源配置策略通过RL解决这一问题存在三个关键挑战：（1）现实世界中复杂的情况和无数的决策选择(2） 由于大流行传播的潜伏期，只有不完善的信息可用(3） 在现实世界中进行实验的局限性，因为我们不能随意设定流行病爆发。本文提出了一种分层强化学习方法，并给出了相应的训练算法。我们设计了一个分解的动作空间来处理无数的选择，以确保有效和实时的策略。我们还设计了一个基于递归神经网络的框架来利用从环境中获得的不完美信息。我们建立了一个基于真实世界数据的大流行传播模拟器，作为实验平台。我们进行了大量实验，结果表明，我们的方法优于所有基线，平均减少感染和死亡14.25%。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AuTO: Scaling Deep Reinforcement Learning for Datacenter-Scale Automatic Tra_x001B_ic Optimization</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>chenkai 老师的文章</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1317,6 +1325,14 @@
         <v>68</v>
       </c>
     </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>94</v>
+      </c>
+      <c r="G20" t="s">
+        <v>95</v>
+      </c>
+    </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>7</v>

</xml_diff>